<commit_message>
feat: implement patient notification email workflow and logging system
</commit_message>
<xml_diff>
--- a/Data/Log_Robot.xlsx
+++ b/Data/Log_Robot.xlsx
@@ -1,141 +1,178 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="1" state="visible" r:id="rId1"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:workbookPr codeName="ThisWorkbook"/>
+  <x:workbookProtection/>
+  <x:bookViews>
+    <x:workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </x:bookViews>
+  <x:sheets>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="1" r:id="rId1"/>
+  </x:sheets>
+  <x:definedNames/>
+  <x:calcPr calcId="124519" fullCalcOnLoad="1"/>
+</x:workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:si>
+    <x:t>27/04/2026 11:09:42</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Karim Gharbi</x:t>
+  </x:si>
+  <x:si>
+    <x:t>16/04/2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>09:30</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Email Envoyé</x:t>
+  </x:si>
+  <x:si>
+    <x:t>27/04/2026 11:11:13</x:t>
+  </x:si>
+</x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-  </fonts>
-  <fills count="3">
-    <fill>
-      <patternFill/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0037474F"/>
-      </patternFill>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
-</styleSheet>
+<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="0"/>
+  <x:fonts count="3">
+    <x:font>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+      <x:color theme="1"/>
+      <x:sz val="11"/>
+      <x:scheme val="minor"/>
+    </x:font>
+    <x:font>
+      <x:name val="Calibri"/>
+      <x:b val="1"/>
+      <x:color rgb="00FFFFFF"/>
+      <x:sz val="11"/>
+    </x:font>
+    <x:font>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+    </x:font>
+  </x:fonts>
+  <x:fills count="3">
+    <x:fill>
+      <x:patternFill patternType="none"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="0037474F"/>
+      </x:patternFill>
+    </x:fill>
+  </x:fills>
+  <x:borders count="1">
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+  </x:borders>
+  <x:cellStyleXfs count="2">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+  </x:cellStyleXfs>
+  <x:cellXfs count="3">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+  </x:cellXfs>
+  <x:cellStyles count="1">
+    <x:cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </x:cellStyles>
+  <x:tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <x:colors>
+    <x:indexedColors>
+      <x:rgbColor rgb="00000000"/>
+      <x:rgbColor rgb="00FFFFFF"/>
+      <x:rgbColor rgb="00FF0000"/>
+      <x:rgbColor rgb="0000FF00"/>
+      <x:rgbColor rgb="000000FF"/>
+      <x:rgbColor rgb="00FFFF00"/>
+      <x:rgbColor rgb="00FF00FF"/>
+      <x:rgbColor rgb="0000FFFF"/>
+      <x:rgbColor rgb="00000000"/>
+      <x:rgbColor rgb="00FFFFFF"/>
+      <x:rgbColor rgb="00FF0000"/>
+      <x:rgbColor rgb="0000FF00"/>
+      <x:rgbColor rgb="000000FF"/>
+      <x:rgbColor rgb="00FFFF00"/>
+      <x:rgbColor rgb="00FF00FF"/>
+      <x:rgbColor rgb="0000FFFF"/>
+      <x:rgbColor rgb="00800000"/>
+      <x:rgbColor rgb="00008000"/>
+      <x:rgbColor rgb="00000080"/>
+      <x:rgbColor rgb="00808000"/>
+      <x:rgbColor rgb="00800080"/>
+      <x:rgbColor rgb="00008080"/>
+      <x:rgbColor rgb="00C0C0C0"/>
+      <x:rgbColor rgb="00808080"/>
+      <x:rgbColor rgb="009999FF"/>
+      <x:rgbColor rgb="00993366"/>
+      <x:rgbColor rgb="00FFFFCC"/>
+      <x:rgbColor rgb="00CCFFFF"/>
+      <x:rgbColor rgb="00660066"/>
+      <x:rgbColor rgb="00FF8080"/>
+      <x:rgbColor rgb="000066CC"/>
+      <x:rgbColor rgb="00CCCCFF"/>
+      <x:rgbColor rgb="00000080"/>
+      <x:rgbColor rgb="00FF00FF"/>
+      <x:rgbColor rgb="00FFFF00"/>
+      <x:rgbColor rgb="0000FFFF"/>
+      <x:rgbColor rgb="00800080"/>
+      <x:rgbColor rgb="00800000"/>
+      <x:rgbColor rgb="00008080"/>
+      <x:rgbColor rgb="000000FF"/>
+      <x:rgbColor rgb="0000CCFF"/>
+      <x:rgbColor rgb="00CCFFFF"/>
+      <x:rgbColor rgb="00CCFFCC"/>
+      <x:rgbColor rgb="00FFFF99"/>
+      <x:rgbColor rgb="0099CCFF"/>
+      <x:rgbColor rgb="00FF99CC"/>
+      <x:rgbColor rgb="00CC99FF"/>
+      <x:rgbColor rgb="00FFCC99"/>
+      <x:rgbColor rgb="003366FF"/>
+      <x:rgbColor rgb="0033CCCC"/>
+      <x:rgbColor rgb="0099CC00"/>
+      <x:rgbColor rgb="00FFCC00"/>
+      <x:rgbColor rgb="00FF9900"/>
+      <x:rgbColor rgb="00FF6600"/>
+      <x:rgbColor rgb="00666699"/>
+      <x:rgbColor rgb="00969696"/>
+      <x:rgbColor rgb="00003366"/>
+      <x:rgbColor rgb="00339966"/>
+      <x:rgbColor rgb="00003300"/>
+      <x:rgbColor rgb="00333300"/>
+      <x:rgbColor rgb="00993300"/>
+      <x:rgbColor rgb="00993366"/>
+      <x:rgbColor rgb="00333399"/>
+      <x:rgbColor rgb="00333333"/>
+    </x:indexedColors>
+  </x:colors>
+</x:styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -422,49 +459,86 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Timestamp</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Patient</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Heure</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Statut</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+    <x:pageSetUpPr/>
+  </x:sheetPr>
+  <x:dimension ref="A1:E1"/>
+  <x:sheetFormatPr baseColWidth="8" defaultColWidth="9.139196" defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="2" width="22" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:5">
+      <x:c r="A1" s="2" t="inlineStr">
+        <x:is>
+          <x:t>Timestamp</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B1" s="2" t="inlineStr">
+        <x:is>
+          <x:t>Patient</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C1" s="2" t="inlineStr">
+        <x:is>
+          <x:t>Date</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D1" s="2" t="inlineStr">
+        <x:is>
+          <x:t>Heure</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E1" s="2" t="inlineStr">
+        <x:is>
+          <x:t>Statut</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:5">
+      <x:c r="A2" s="0" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:5">
+      <x:c r="A3" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
[AMELORATION] feat: implement patient appointment confirmation email notification workflow
</commit_message>
<xml_diff>
--- a/Data/Log_Robot.xlsx
+++ b/Data/Log_Robot.xlsx
@@ -39,6 +39,15 @@
   </x:si>
   <x:si>
     <x:t>27/04/2026 11:27:49</x:t>
+  </x:si>
+  <x:si>
+    <x:t>27/04/2026 15:20:03</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Laith Mahdi</x:t>
+  </x:si>
+  <x:si>
+    <x:t>27/04/2026 15:23:18</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -574,6 +583,40 @@
         <x:v>4</x:v>
       </x:c>
     </x:row>
+    <x:row r="6" spans="1:5">
+      <x:c r="A6" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:5">
+      <x:c r="A7" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: implement LireDemandesExcel workflow to process pending patient appointment requests from Excel
</commit_message>
<xml_diff>
--- a/Data/Log_Robot.xlsx
+++ b/Data/Log_Robot.xlsx
@@ -48,6 +48,21 @@
   </x:si>
   <x:si>
     <x:t>27/04/2026 15:23:18</x:t>
+  </x:si>
+  <x:si>
+    <x:t>27/04/2026 15:26:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>27/04/2026 15:29:06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>27/04/2026 15:34:27</x:t>
+  </x:si>
+  <x:si>
+    <x:t>habib razeg</x:t>
+  </x:si>
+  <x:si>
+    <x:t>27/04/2026 15:36:26</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -617,6 +632,74 @@
         <x:v>4</x:v>
       </x:c>
     </x:row>
+    <x:row r="8" spans="1:5">
+      <x:c r="A8" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:5">
+      <x:c r="A9" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:5">
+      <x:c r="A10" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E10" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:5">
+      <x:c r="A11" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C11" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E11" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: implement workflow to extract pending patient requests from Excel data file
</commit_message>
<xml_diff>
--- a/Data/Log_Robot.xlsx
+++ b/Data/Log_Robot.xlsx
@@ -37,43 +37,19 @@
     <x:t>Statut</x:t>
   </x:si>
   <x:si>
-    <x:t>27/04/2026 11:09:42</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Karim Gharbi</x:t>
-  </x:si>
-  <x:si>
-    <x:t>16/04/2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>09:30</x:t>
+    <x:t>29/04/2026 14:26:28</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Laith Mahdi</x:t>
+  </x:si>
+  <x:si>
+    <x:t>04/29/2026 00:00:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>15:00:00</x:t>
   </x:si>
   <x:si>
     <x:t>Email Envoyé</x:t>
-  </x:si>
-  <x:si>
-    <x:t>27/04/2026 11:11:13</x:t>
-  </x:si>
-  <x:si>
-    <x:t>27/04/2026 11:26:18</x:t>
-  </x:si>
-  <x:si>
-    <x:t>27/04/2026 11:27:49</x:t>
-  </x:si>
-  <x:si>
-    <x:t>27/04/2026 17:13:55</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Laith Mahdi</x:t>
-  </x:si>
-  <x:si>
-    <x:t>27/04/2026 17:14:55</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Yassine mahdi</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10:00</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -446,7 +422,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:E5"/>
+  <x:dimension ref="A1:E1"/>
   <x:sheetFormatPr defaultColWidth="9.139196" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <x:cols>
     <x:col min="1" max="2" width="22" style="0" customWidth="1"/>
@@ -472,7 +448,7 @@
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <x:row r="2" spans="1:5">
       <x:c r="A2" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -486,91 +462,6 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <x:c r="A3" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D3" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <x:c r="A4" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D4" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <x:c r="A5" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D5" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="E5" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:5">
-      <x:c r="A6" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D6" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="E6" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:5">
-      <x:c r="A7" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D7" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E7" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat: implement appointment availability verification and status update workflows with associated data management
</commit_message>
<xml_diff>
--- a/Data/Log_Robot.xlsx
+++ b/Data/Log_Robot.xlsx
@@ -1,146 +1,120 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15">
-  <x:fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <x:workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mahdi\OneDrive\Documents\mini-project-rpa\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11820" firstSheet="0" activeTab="0"/>
-  </x:bookViews>
-  <x:sheets>
-    <x:sheet name="Log" sheetId="1" r:id="rId1"/>
-  </x:sheets>
-  <x:definedNames/>
-  <x:calcPr calcId="0"/>
-</x:workbook>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11820"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Log" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="0"/>
+</workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:si>
-    <x:t>Timestamp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Patient</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Date</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Heure</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Statut</x:t>
-  </x:si>
-  <x:si>
-    <x:t>29/04/2026 14:34:59</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Laith Mahdi</x:t>
-  </x:si>
-  <x:si>
-    <x:t>04/29/2026 00:00:00</x:t>
-  </x:si>
-  <x:si>
-    <x:t>15:00:00</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Email Envoyé</x:t>
-  </x:si>
-  <x:si>
-    <x:t>29/04/2026 14:37:35</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Dalel Loussaief</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11:00</x:t>
-  </x:si>
-</x:sst>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>Timestamp</t>
+  </si>
+  <si>
+    <t>Patient</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Heure</t>
+  </si>
+  <si>
+    <t>Statut</t>
+  </si>
+  <si>
+    <t>29/04/2026 14:34:59</t>
+  </si>
+  <si>
+    <t>Laith Mahdi</t>
+  </si>
+  <si>
+    <t>04/29/2026 00:00:00</t>
+  </si>
+  <si>
+    <t>15:00:00</t>
+  </si>
+  <si>
+    <t>Email Envoyé</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac x16r2">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="3" x14ac:knownFonts="1">
-    <x:font>
-      <x:sz val="11"/>
-      <x:color theme="1"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-      <x:scheme val="minor"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="3">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF37474F"/>
-      </x:patternFill>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="2">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="3">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-  <x:tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <x:extLst>
-    <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+  </fonts>
+  <fills count="3">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF37474F"/>
+      </patternFill>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </x:ext>
-    <x:ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
       <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </x:ext>
-  </x:extLst>
-</x:styleSheet>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -427,75 +401,51 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
-  <x:sheetPr>
-    <x:outlinePr summaryBelow="1" summaryRight="1"/>
-  </x:sheetPr>
-  <x:dimension ref="A1:E1"/>
-  <x:sheetFormatPr defaultColWidth="9.139196" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <x:cols>
-    <x:col min="1" max="2" width="22" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="12" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="8" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" style="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <x:c r="A1" s="2" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B1" s="2" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E1" s="2" t="s">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:5">
-      <x:c r="A2" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B2" s="0" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C2" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D2" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="E2" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:5">
-      <x:c r="A3" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D3" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
-  <x:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
-  <x:headerFooter/>
-  <x:tableParts count="0"/>
-</x:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add API documentation and improve server functionality
- Created contributing guidelines and issue reporting documentation.
- Added CLI usage instructions for swagger-jsdoc.
- Integrated Swagger UI for API documentation in the server.
- Defined OpenAPI specifications for login and appointment endpoints.
- Enhanced appointment retrieval logic with detailed response structure.
- Implemented error handling for data reading and writing operations.

Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/Data/Log_Robot.xlsx
+++ b/Data/Log_Robot.xlsx
@@ -1,120 +1,146 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<x:workbook xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15">
+  <x:fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <x:workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mahdi\OneDrive\Documents\mini-project-rpa\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11820"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Log" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="0"/>
-</workbook>
+  <x:bookViews>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11820" firstSheet="0" activeTab="0"/>
+  </x:bookViews>
+  <x:sheets>
+    <x:sheet name="Log" sheetId="1" r:id="rId1"/>
+  </x:sheets>
+  <x:definedNames/>
+  <x:calcPr calcId="0"/>
+</x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>Timestamp</t>
-  </si>
-  <si>
-    <t>Patient</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Heure</t>
-  </si>
-  <si>
-    <t>Statut</t>
-  </si>
-  <si>
-    <t>29/04/2026 14:34:59</t>
-  </si>
-  <si>
-    <t>Laith Mahdi</t>
-  </si>
-  <si>
-    <t>04/29/2026 00:00:00</t>
-  </si>
-  <si>
-    <t>15:00:00</t>
-  </si>
-  <si>
-    <t>Email Envoyé</t>
-  </si>
-</sst>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:si>
+    <x:t>Timestamp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Patient</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Date</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Heure</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Statut</x:t>
+  </x:si>
+  <x:si>
+    <x:t>29/04/2026 14:34:59</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Laith Mahdi</x:t>
+  </x:si>
+  <x:si>
+    <x:t>04/29/2026 00:00:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>15:00:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Email Envoyé</x:t>
+  </x:si>
+  <x:si>
+    <x:t>29/04/2026 14:49:42</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Mahdi Leith</x:t>
+  </x:si>
+  <x:si>
+    <x:t>15:30:00</x:t>
+  </x:si>
+</x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-  </fonts>
-  <fills count="3">
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF37474F"/>
-      </patternFill>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+<x:styleSheet xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac x16r2">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="0" formatCode=""/>
+  </x:numFmts>
+  <x:fonts count="3" x14ac:knownFonts="1">
+    <x:font>
+      <x:sz val="11"/>
+      <x:color theme="1"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+    </x:font>
+  </x:fonts>
+  <x:fills count="3">
+    <x:fill>
+      <x:patternFill patternType="none"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF37474F"/>
+      </x:patternFill>
+    </x:fill>
+  </x:fills>
+  <x:borders count="1">
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+  </x:borders>
+  <x:cellStyleXfs count="2">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+  </x:cellStyleXfs>
+  <x:cellXfs count="3">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+  </x:cellXfs>
+  <x:cellStyles count="1">
+    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </x:cellStyles>
+  <x:tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <x:extLst>
+    <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+    </x:ext>
+    <x:ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
       <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
-</styleSheet>
+    </x:ext>
+  </x:extLst>
+</x:styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -401,51 +427,75 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="8" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:E2"/>
+  <x:sheetFormatPr defaultColWidth="9.139196" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <x:cols>
+    <x:col min="1" max="2" width="22" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <x:c r="A1" s="2" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="2" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C1" s="2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1" s="2" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1" s="2" t="s">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <x:c r="A2" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:5">
+      <x:c r="A3" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
 </file>
</xml_diff>